<commit_message>
Add images for remaining 23 markers, re-create migration page
All 50 markers now have CC-licensed photos from Wikimedia Commons.
10 new flagged entries added to spreadsheet for approximate images.
Migration page re-created for uploading to Firebase Storage.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/flagged-marker-images.xlsx
+++ b/flagged-marker-images.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Flagged Images" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flagged Images'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flagged Images'!$A$1:$D$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -583,8 +583,228 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>CW17</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Crickley Hill</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Car park at Crickley Hill Country Park</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Shows the car park area, not the hill viewpoint itself</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>CW21</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Cranham Corner</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>View of Cranham village from the east</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>General village view, not the specific trail marker corner</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>CW24</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Edge Village</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Mid-Cotswolds landscape near Edge</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Landscape near Edge, not the village itself</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>CW26</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Scottsquar Hill</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Quarry on Scottsquar Hill</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Shows a quarry on the hill, not the trail viewpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>CW29</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Uley Bury</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Uley village below Uley Bury</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>View of the village from below, not from the hillfort</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>CW36</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Hawkesbury Upton</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Hawkesbury Upton war memorial</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>War memorial, not the wider village or trail marker</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>CW40</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Dodington Park Gate</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Bath Lodge at Dodington Park</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Shows Bath Lodge entrance, not the specific gate on the trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>CW43</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Pennsylvania</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>View south towards Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Distant landscape view toward the area</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>CW44</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Cold Ashton Village</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Cold Ashton village green</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Generic village green view, may not match marker location</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>CW47</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Prospect Stile, Lansdown</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Grenville Monument on Lansdown Battlefield</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Shows nearby monument, not the Prospect Stile viewpoint</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D6"/>
+  <autoFilter ref="A1:D16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>